<commit_message>
HBM v0.5.1: verify Ascend 950PR memory (official 'low-cost HBM' HiBL 1.0; Atlas 350 112GB/1.4TB/s; Reuters: base version DDR; Epoch LPDDR inference; no teardown), evidence table with tiers, sources 90-97, prediction C8; China ledger base unchanged with sensitivity
</commit_message>
<xml_diff>
--- a/hbm/hbm_model.xlsx
+++ b/hbm/hbm_model.xlsx
@@ -3040,7 +3040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Epoch AI 2026-09（09-24 更新）《Huawei’s roadmap to 2031》：华为 2025 年约 80 万、2026 年中位约 150 万（950PR 约 75 万用类 LPDDR 非 HBM、910C 约 43 万用囤货、950DT 约 24 万用长鑫+武汉新芯 HBM、约 8 万用走私 HBM）；囤货多为 8 层 HBM2E 16GB、2026 年用完；长鑫 HBM 投片沿用 SemiAnalysis 口径、武汉新芯约为长鑫 1/10；北方华创 2026-03 发布混合键合机；TSV 刻蚀部分受控（Lam 受控、TEL 不受控）</t>
+          <t>Epoch AI 2026-09（09-24 更新）《Huawei’s roadmap to 2031》：华为 2025 年约 80 万、2026 年中位约 150 万（950PR 约 75 万"可能"用接近 LPDDR 的非 HBM 内存（Epoch 依据一张疑似芯片照片推测：内存模块离计算 die 太远，不像 HBM）、910C 约 43 万用囤货、950DT 约 24 万用长鑫+武汉新芯 HBM、约 8 万用走私 HBM）；囤货多为 8 层 HBM2E 16GB、2026 年用完；长鑫 HBM 投片沿用 SemiAnalysis 口径、武汉新芯约为长鑫 1/10；北方华创 2026-03 发布混合键合机；TSV 刻蚀部分受控（Lam 受控、TEL 不受控）</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>华为 2025-09-18 全联接大会徐直军主题演讲：950PR（自研 HiBL 1.0，128GB、1.6TB/s，2026Q1）、950DT（HiZQ 2.0，144GB、4TB/s，2026Q4）、960（2027Q4）、970（2028Q4）</t>
+          <t>华为 2025-09-18 全联接大会徐直军主题演讲（官方文字稿）：950 系列配两种自研 HBM，"与 Ascend 950 Die 合封"；HiBL 1.0 是"自研低成本 HBM，比 HBM3E/HBM4E 更划算"（950PR，2026Q1）；HiZQ 2.0 为 144GB、4TB/s（950DT，2026Q4）；960（2027Q4）、970（2028Q4）。注意：950PR 的 128GB、1.6TB/s 不在文字稿里，见发布会幻灯片转述（路透、Tom’s Hardware）与昇腾官网（源90）</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4392,6 +4392,126 @@
       <c r="C90" t="inlineStr">
         <is>
           <t>https://caifuhao.eastmoney.com/news/20260527190247307266190</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>昇腾官网 Ascend 950PR 处理器页：最大配备 128GB、1.6TB/s"高速片上内存"（页面未写 HBM）</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://www.hiascend.com/hardware/processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>昇腾官网 Atlas 350 加速卡（950PR）技术规格：内存 112 GB HBM、带宽 1.4TB/s、支持 ECC，最大功耗 ≤600W</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://www.hiascend.com/hardware/accelerator-card</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>路透 2026-03-27 独家（RTHK 转载）：华为 2026 年计划出货约 75 万颗 950PR，4 月量产、下半年放量；用传统 DDR 内存的版本约 5 万元/卡，用更快 HBM 的高配版约 7 万元</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://news.rthk.hk/rthk/en/component/k2/1849055-20260327.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Business Times（转引彭博）2025-10：TechInsights 拆解多枚 910C，发现台积电代工的 die，以及三星、SK 海力士的 HBM2E（分别出现在两个不同样本里）；台积电称这些 die 与 2024-10 分析过的是同一批</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://www.businesstimes.com.sg/companies-markets/huawei-used-tsmc-samsung-sk-hynix-components-top-ai-chips-techinsights</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>heise 2024-10：TechInsights 拆解 Atlas 300T A2 加速卡中的昇腾 910B，发现台积电制造的芯片</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://www.heise.de/en/news/Surprise-TSMC-technology-found-in-Huawei-s-AI-accelerator-9992277.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>TechPowerUp 2025-12：昇腾 950 芯片照片首次曝光，作者称计算 die 周围的内存"像 LPDDR/HBM 混合体"（照片判读，非拆解）</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://www.techpowerup.com/344062/huawei-ascend-950-ai-accelerator-pictured</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Huawei Central 2026-07-03（转引 X 用户 @zephyr_z9 泄露图）：950PR 封装为 2 个 AI die + 8 个内存模块，950DT 为 4 个 HiZQ 堆栈、每堆栈约 1TB/s（泄露，未证实；网站拒绝 curl，据搜索摘要）</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://www.huaweicentral.com/huawei-ascend-950dt-die-chip-design-details/</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Tom's Hardware 2026-03：Atlas 350 配 112GB 华为自研 HiBL 1.0、1.4TB/s；内存供应商未知</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/pc-components/gpus/huawei-unveils-new-atlas-350-ai-accelerator-with-1-56-pflops-of-fp4-compute-and-up-to-112gb-of-hbm-claims-2-8x-more-performance-than-nvidias-h20</t>
         </is>
       </c>
     </row>

</xml_diff>